<commit_message>
data: 更新 2026-03 (TT=192.846 Kwai=65.057)
</commit_message>
<xml_diff>
--- a/docs/data/巴西数据底稿_2026-03.xlsx
+++ b/docs/data/巴西数据底稿_2026-03.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026_03" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="未分类App" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026_03" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="未分类App" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -505,19 +505,19 @@
     </row>
     <row r="2">
       <c r="B2" t="n">
-        <v>393.84</v>
+        <v>394.57</v>
       </c>
       <c r="C2" t="n">
-        <v>507.01</v>
+        <v>519.1799999999999</v>
       </c>
       <c r="D2" t="n">
         <v>1.37</v>
       </c>
       <c r="E2" t="n">
-        <v>291.62</v>
+        <v>291.78</v>
       </c>
       <c r="F2" t="n">
-        <v>13.4</v>
+        <v>16.96</v>
       </c>
       <c r="G2" t="n">
         <v>0.71</v>
@@ -526,7 +526,7 @@
         <v>7.8</v>
       </c>
       <c r="I2" t="n">
-        <v>98.13</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="J2" t="n">
         <v>20.85</v>
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>183.219</v>
+        <v>192.846</v>
       </c>
     </row>
     <row r="11">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>62.52</v>
+        <v>65.057</v>
       </c>
     </row>
     <row r="12">
@@ -734,424 +734,434 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>waze</t>
+          <t>Waze</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>11.891</v>
+        <v>9.318</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>Pinterest</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1.501</v>
+        <v>6.135</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Quora</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.008</v>
+        <v>1.501</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Quora</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0.008</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Helo - Share Your Life</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F30" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Google News</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>0.171</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>Google News</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>0.138</v>
+        <v>0.171</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>UOL | Notícias em Tempo Real</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0.074</v>
+        <v>0.138</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Panflix</t>
+          <t>UOL | Notícias em Tempo Real</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.064</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Panflix</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0.064</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Zero Hora</t>
         </is>
       </c>
-      <c r="G35" t="n">
+      <c r="G36" t="n">
         <v>0.018</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Wattpad</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>1.746</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kindle</t>
+          <t>Wattpad</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.065</v>
+        <v>1.746</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>JW Library</t>
+          <t>Kindle</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>0.832</v>
+        <v>1.065</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GALATEA</t>
+          <t>JW Library</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.674</v>
+        <v>0.832</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>GALATEA</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>0.674</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Bible</t>
         </is>
       </c>
-      <c r="H41" t="n">
+      <c r="H42" t="n">
         <v>0.419</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Chrome Browser</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>60.965</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Chrome Browser</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>24.926</v>
+        <v>60.965</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Brave Browser: Fast AdBlocker</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>3.672</v>
+        <v>24.926</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Seekee - Safe&amp;Fast Browser</t>
+          <t>Brave Browser: Fast AdBlocker</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>2.23</v>
+        <v>3.672</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Seekee - Safe&amp;Fast Browser</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>2.23</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>Samsung Internet Browser</t>
         </is>
       </c>
-      <c r="I47" t="n">
+      <c r="I48" t="n">
         <v>2.109</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Spotify</t>
-        </is>
-      </c>
-      <c r="J49" t="n">
-        <v>10.432</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>YouTube Music</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>4.716</v>
+        <v>10.432</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Lark Player</t>
+          <t>YouTube Music</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>0.947</v>
+        <v>4.716</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mi Music</t>
+          <t>Lark Player</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>0.474</v>
+        <v>0.947</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Mi Music</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>0.474</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>Music Player - MP3 Player, Audio Player</t>
         </is>
       </c>
-      <c r="J53" t="n">
+      <c r="J54" t="n">
         <v>0.233</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ROBLOX</t>
-        </is>
-      </c>
-      <c r="K55" t="n">
-        <v>38.488</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Brawl Stars</t>
+          <t>ROBLOX</t>
         </is>
       </c>
       <c r="K56" t="n">
-        <v>6.552</v>
+        <v>38.488</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Free Fire</t>
+          <t>Brawl Stars</t>
         </is>
       </c>
       <c r="K57" t="n">
-        <v>6.303</v>
+        <v>6.552</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Clash Royale</t>
+          <t>Free Fire</t>
         </is>
       </c>
       <c r="K58" t="n">
-        <v>3.63</v>
+        <v>6.303</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>Clash Royale</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>3.63</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Minecraft Pocket Edition</t>
         </is>
       </c>
-      <c r="K59" t="n">
+      <c r="K60" t="n">
         <v>3.342</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Shopee</t>
-        </is>
-      </c>
-      <c r="L61" t="n">
-        <v>14.512</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MercadoLibre</t>
+          <t>Shopee</t>
         </is>
       </c>
       <c r="L62" t="n">
-        <v>6.525</v>
+        <v>14.512</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SHEIN</t>
+          <t>MercadoLibre</t>
         </is>
       </c>
       <c r="L63" t="n">
-        <v>2.806</v>
+        <v>6.525</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>SHEIN</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>1.323</v>
+        <v>2.806</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>1.323</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>OLX Brasil</t>
         </is>
       </c>
-      <c r="L65" t="n">
+      <c r="L66" t="n">
         <v>1.049</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Uber</t>
-        </is>
-      </c>
-      <c r="M67" t="n">
-        <v>2.675</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>99Taxis</t>
+          <t>Uber</t>
         </is>
       </c>
       <c r="M68" t="n">
-        <v>2.577</v>
+        <v>2.675</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>iFood Delivery de Comida</t>
+          <t>99Taxis</t>
         </is>
       </c>
       <c r="M69" t="n">
-        <v>2.41</v>
+        <v>2.577</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>iFood Delivery de Comida</t>
         </is>
       </c>
       <c r="M70" t="n">
-        <v>0.432</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>0.432</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
           <t>inDrive</t>
         </is>
       </c>
-      <c r="M71" t="n">
+      <c r="M72" t="n">
         <v>0.347</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>其他</t>
         </is>
       </c>
-      <c r="B73" t="n">
-        <v>17.466</v>
-      </c>
-      <c r="E73" t="n">
-        <v>3.195</v>
-      </c>
-      <c r="G73" t="n">
+      <c r="B74" t="n">
+        <v>18.196</v>
+      </c>
+      <c r="E74" t="n">
+        <v>3.351</v>
+      </c>
+      <c r="G74" t="n">
         <v>0.242</v>
       </c>
-      <c r="H73" t="n">
+      <c r="H74" t="n">
         <v>3.06</v>
       </c>
-      <c r="I73" t="n">
-        <v>4.228</v>
-      </c>
-      <c r="J73" t="n">
+      <c r="I74" t="n">
+        <v>4.247</v>
+      </c>
+      <c r="J74" t="n">
         <v>4.044</v>
       </c>
-      <c r="K73" t="n">
+      <c r="K74" t="n">
         <v>63.674</v>
       </c>
-      <c r="L73" t="n">
+      <c r="L74" t="n">
         <v>3.959</v>
       </c>
-      <c r="M73" t="n">
+      <c r="M74" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1166,7 +1176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1228,580 +1238,540 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Waze</t>
+          <t>POCO Launcher 2.0 - Customize,</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9.318</v>
+        <v>7.15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>POCO Launcher 2.0 - Customize,</t>
+          <t>Emochi: Unlimited Chat with AI</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.15</v>
+        <v>5.968</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pinterest</t>
+          <t>Google Maps</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.135</v>
+        <v>5.235</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Emochi: Unlimited Chat with AI</t>
+          <t>Phone by Google</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5.968</v>
+        <v>3.978</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Character AI</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5.235</v>
+        <v>3.864</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Phone by Google</t>
+          <t>OiTube</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.978</v>
+        <v>3.321</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Character AI</t>
+          <t>YouTube Kids</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3.864</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OiTube</t>
+          <t>Uber Driver</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.321</v>
+        <v>3.065</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>YouTube Kids</t>
+          <t>99 POP</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.16</v>
+        <v>2.992</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Uber Driver</t>
+          <t>Nubank</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.065</v>
+        <v>2.889</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>99 POP</t>
+          <t>Duolingo: Learn Languages</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.992</v>
+        <v>2.789</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nubank</t>
+          <t>ibisPaint</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.889</v>
+        <v>2.533</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Duolingo: Learn Languages</t>
+          <t>Melolo - Short Movie &amp; TV</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.789</v>
+        <v>2.508</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ibisPaint</t>
+          <t>Samsung Clock</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2.533</v>
+        <v>2.156</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Melolo - Short Movie &amp; TV</t>
+          <t>Itaú</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2.508</v>
+        <v>2.153</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Samsung Clock</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2.156</v>
+        <v>2.064</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Itaú</t>
+          <t>Google Drive</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2.153</v>
+        <v>2.011</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Microsoft Teams</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2.064</v>
+        <v>1.899</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Google Drive</t>
+          <t>DramaReels - Pure Short Dramas</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.011</v>
+        <v>1.867</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Microsoft Teams</t>
+          <t>Tomato - A&amp;M</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1.899</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DramaReels - Pure Short Dramas</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1.867</v>
+        <v>1.527</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tomato - A&amp;M</t>
+          <t>CAIXA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1.71</v>
+        <v>1.402</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>Banco do Brasil</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1.527</v>
+        <v>1.238</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>Santander Brasil</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1.402</v>
+        <v>1.229</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Disney+</t>
+          <t>Bradesco</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.256</v>
+        <v>1.202</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Banco do Brasil</t>
+          <t>Calculator by Google</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1.238</v>
+        <v>1.165</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Santander Brasil</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.229</v>
+        <v>1.126</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bradesco</t>
+          <t>Files Go by Google</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1.202</v>
+        <v>1.087</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Calculator by Google</t>
+          <t>SnapTube</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.165</v>
+        <v>1.049</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>FuzzTv</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1.126</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Files Go by Google</t>
+          <t>Google Play services</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1.087</v>
+        <v>1.026</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SnapTube</t>
+          <t>Microsoft Outlook</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1.049</v>
+        <v>1.017</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FuzzTv</t>
+          <t>PicPay</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1.043</v>
+        <v>0.965</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Google Play services</t>
+          <t>Crunchyroll</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1.026</v>
+        <v>0.911</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Microsoft Outlook</t>
+          <t>GreenTuber block ads on videos</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1.017</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PicPay</t>
+          <t>Banco Inter</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.965</v>
+        <v>0.887</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Crunchyroll</t>
+          <t>Sua Novela - Drama Grátis</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.911</v>
+        <v>0.8159999999999999</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GreenTuber block ads on videos</t>
+          <t>Dootchi: Chat with AI Chars</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.895</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Banco Inter</t>
+          <t>Cici</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.887</v>
+        <v>0.769</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sua Novela - Drama Grátis</t>
+          <t>Canva</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.761</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dootchi: Chat with AI Chars</t>
+          <t>Glance</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.8</v>
+        <v>0.758</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Cici</t>
+          <t>Grok - AI Assistant</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.769</v>
+        <v>0.737</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Canva</t>
+          <t>Adobe Reader</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.761</v>
+        <v>0.707</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Glance</t>
+          <t>iCSee</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.758</v>
+        <v>0.694</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Grok - AI Assistant</t>
+          <t>Nova Launcher</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.737</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tinder</t>
+          <t>Google Docs</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.73</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Adobe Reader</t>
+          <t>Android Auto</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.707</v>
+        <v>0.677</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>iCSee</t>
+          <t>Samsung Calculator</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.694</v>
+        <v>0.655</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Nova Launcher</t>
+          <t>Samsung Notes</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.627</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Google Docs</t>
+          <t>Saylo</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.679</v>
+        <v>0.607</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Android Auto</t>
+          <t>XOS Launcher -Cool Stylish</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.677</v>
+        <v>0.556</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Samsung Calculator</t>
+          <t>ZOOM Cloud Meetings</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.655</v>
+        <v>0.552</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Samsung Notes</t>
+          <t>Entregador</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.627</v>
+        <v>0.532</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Saylo</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.607</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>XOS Launcher -Cool Stylish</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>0.556</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>ZOOM Cloud Meetings</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>0.552</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Entregador</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>0.532</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
         <v>0.524</v>
       </c>
     </row>

</xml_diff>